<commit_message>
fix: update environment variable loading for Supabase integration and remove temporary Excel file
</commit_message>
<xml_diff>
--- a/Chia nhiệm vụ dự án MentorPro.xlsx
+++ b/Chia nhiệm vụ dự án MentorPro.xlsx
@@ -1,17 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MentorPro\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0836151C-BC48-4D4E-89B2-DB00E9053193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Chia nhiệm vụ dự án MentorPro" sheetId="1" r:id="rId5"/>
+    <sheet name="Chia nhiệm vụ dự án MentorPro" sheetId="1" r:id="rId1"/>
+    <sheet name="Checklist Dự án MentorPro" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="70">
   <si>
     <t>Thành viên</t>
   </si>
@@ -68,35 +78,215 @@
   </si>
   <si>
     <t>* Triển khai dự án lên máy ảo (Render cho Backend, Vercel cho Frontend).* Quản lý bảo mật file .env trên môi trường Production.* Viết tài liệu hướng dẫn (README) và thực hiện các kịch bản test lỗi.</t>
+  </si>
+  <si>
+    <t>Hạng mục</t>
+  </si>
+  <si>
+    <t>Công việc</t>
+  </si>
+  <si>
+    <t>Chi tiết</t>
+  </si>
+  <si>
+    <t>Kiến trúc &amp; Khởi tạo</t>
+  </si>
+  <si>
+    <t>Chốt Tech Stack</t>
+  </si>
+  <si>
+    <t>Next.js, FastAPI, Supabase, Gemini API</t>
+  </si>
+  <si>
+    <t>Hoàn thành</t>
+  </si>
+  <si>
+    <t>Cấu trúc thư mục</t>
+  </si>
+  <si>
+    <t>Tạo folder frontend/ và backend/</t>
+  </si>
+  <si>
+    <t>Git &amp; GitHub</t>
+  </si>
+  <si>
+    <t>Khởi tạo repo, .gitignore, kết nối GitHub</t>
+  </si>
+  <si>
+    <t>Backend</t>
+  </si>
+  <si>
+    <t>Môi trường ảo</t>
+  </si>
+  <si>
+    <t>Thiết lập venv</t>
+  </si>
+  <si>
+    <t>Cài đặt thư viện</t>
+  </si>
+  <si>
+    <t>Cài đặt core libraries (FastAPI, Gemini, Pillow, v.v.)</t>
+  </si>
+  <si>
+    <t>Xử lý lỗi C++</t>
+  </si>
+  <si>
+    <t>Sử dụng Pre-compiled Wheels</t>
+  </si>
+  <si>
+    <t>Logic xử lý (main.py)</t>
+  </si>
+  <si>
+    <t>Chatbot và OCR (đọc ảnh)</t>
+  </si>
+  <si>
+    <t>Database</t>
+  </si>
+  <si>
+    <t>Khởi tạo Supabase</t>
+  </si>
+  <si>
+    <t>Tạo dự án MentorPro trên Supabase</t>
+  </si>
+  <si>
+    <t>Cấu trúc bảng (SQL)</t>
+  </si>
+  <si>
+    <t>Tạo bảng messages và thiết lập RLS</t>
+  </si>
+  <si>
+    <t>Kết nối hệ thống</t>
+  </si>
+  <si>
+    <t>Backend &lt;-&gt; Database</t>
+  </si>
+  <si>
+    <t>Kiểm thử lưu trữ tin nhắn thực tế</t>
+  </si>
+  <si>
+    <t>Authentication</t>
+  </si>
+  <si>
+    <t>Google Auth Setup</t>
+  </si>
+  <si>
+    <t>Lấy Client ID/Secret từ Google Cloud Console</t>
+  </si>
+  <si>
+    <t>Frontend</t>
+  </si>
+  <si>
+    <t>Giao diện Chat</t>
+  </si>
+  <si>
+    <t>Xây dựng UI với Tailwind CSS</t>
+  </si>
+  <si>
+    <t>Xử lý Clipboard (onPaste)</t>
+  </si>
+  <si>
+    <t>Dán ảnh trực tiếp từ clipboard</t>
+  </si>
+  <si>
+    <t>Kết nối API</t>
+  </si>
+  <si>
+    <t>Liên kết UI với Backend (/chat</t>
+  </si>
+  <si>
+    <t>/ocr)</t>
+  </si>
+  <si>
+    <t>Tích hợp Đăng nhập</t>
+  </si>
+  <si>
+    <t>Nút Login Google và quản lý user_id</t>
+  </si>
+  <si>
+    <t>Deployment</t>
+  </si>
+  <si>
+    <t>Triển khai Backend</t>
+  </si>
+  <si>
+    <t>Đưa lên Render/Railway</t>
+  </si>
+  <si>
+    <t>Triển khai Frontend</t>
+  </si>
+  <si>
+    <t>Đưa lên Vercel</t>
+  </si>
+  <si>
+    <t>Cấu hình máy ảo</t>
+  </si>
+  <si>
+    <t>Thiết lập .env trên VPS/Cloud</t>
+  </si>
+  <si>
+    <t>Kiểm thử</t>
+  </si>
+  <si>
+    <t>Testing &amp; QA</t>
+  </si>
+  <si>
+    <t>Kiểm tra các trường hợp biên, lỗi AI, auth</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF93C47D"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
-  <borders count="2">
-    <border/>
+  <borders count="3">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -110,29 +300,52 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -140,7 +353,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -330,22 +543,26 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="10.63"/>
-    <col customWidth="1" min="2" max="2" width="21.75"/>
-    <col customWidth="1" min="3" max="3" width="148.38"/>
+    <col min="1" max="1" width="10.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.77734375" customWidth="1"/>
+    <col min="3" max="3" width="168.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36.0" customHeight="1">
+    <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -358,9 +575,9 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" ht="50.25" customHeight="1">
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -373,9 +590,9 @@
       <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" ht="48.0" customHeight="1">
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -388,9 +605,9 @@
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="4" ht="41.25" customHeight="1">
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -400,12 +617,12 @@
       <c r="C4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" ht="36.75" customHeight="1">
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" spans="1:5" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
@@ -418,9 +635,304 @@
       <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="2"/>
+      <c r="E5" s="1"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE36B8C3-337D-4F75-BEDD-54A03575897A}">
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: update project spreadsheet with latest changes
</commit_message>
<xml_diff>
--- a/Chia nhiệm vụ dự án MentorPro.xlsx
+++ b/Chia nhiệm vụ dự án MentorPro.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MentorPro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0836151C-BC48-4D4E-89B2-DB00E9053193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1D208F6-055C-4674-9585-FDDC7CD90F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chia nhiệm vụ dự án MentorPro" sheetId="1" r:id="rId1"/>
@@ -557,7 +557,7 @@
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.6640625" customWidth="1"/>
-    <col min="2" max="2" width="21.77734375" customWidth="1"/>
+    <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="168.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
feat: enhance chat API with rate limiting and chat history retrieval
</commit_message>
<xml_diff>
--- a/Chia nhiệm vụ dự án MentorPro.xlsx
+++ b/Chia nhiệm vụ dự án MentorPro.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MentorPro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1D208F6-055C-4674-9585-FDDC7CD90F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DAB25DF-B9D5-451E-ACA7-613A8A1FED22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chia nhiệm vụ dự án MentorPro" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="69">
   <si>
     <t>Thành viên</t>
   </si>
@@ -191,12 +191,6 @@
     <t>Kết nối API</t>
   </si>
   <si>
-    <t>Liên kết UI với Backend (/chat</t>
-  </si>
-  <si>
-    <t>/ocr)</t>
-  </si>
-  <si>
     <t>Tích hợp Đăng nhập</t>
   </si>
   <si>
@@ -231,6 +225,9 @@
   </si>
   <si>
     <t>Kiểm tra các trường hợp biên, lỗi AI, auth</t>
+  </si>
+  <si>
+    <t>Liên kết UI với Backend (/chat, /ocr)</t>
   </si>
 </sst>
 </file>
@@ -265,7 +262,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -274,7 +271,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF93C47D"/>
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -321,16 +330,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -617,7 +632,7 @@
       <c r="C4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>15</v>
       </c>
       <c r="E4" s="1"/>
@@ -647,9 +662,10 @@
   <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.109375" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" customWidth="1"/>
+    <col min="3" max="3" width="52.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
@@ -667,268 +683,268 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+    <row r="15" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="C16" s="6" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B16" s="2" t="s">
+      <c r="D16" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="B17" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="C17" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B17" s="2" t="s">
+    <row r="18" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C18" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D18" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B18" s="2" t="s">
+    <row r="19" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B19" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C19" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D19" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B19" s="2" t="s">
+    <row r="20" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="B20" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
+      <c r="C20" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="6" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: Update Excel file with new project data
</commit_message>
<xml_diff>
--- a/Chia nhiệm vụ dự án MentorPro.xlsx
+++ b/Chia nhiệm vụ dự án MentorPro.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mã nguồn mở\MentorPro-04339bded746dd3f25dd243e8029613470ca08e3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MentorPro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17FDDE2C-DE5C-4D85-AE99-4FA513EDE6FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{782FD814-F13C-4852-A6A2-8C234B0E133E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chia nhiệm vụ dự án MentorPro" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="65">
   <si>
     <t>Thành viên</t>
   </si>
@@ -29,57 +29,27 @@
     <t>Vai trò</t>
   </si>
   <si>
-    <t>Nhiệm vụ chi tiết (Dựa trên Checklist)</t>
-  </si>
-  <si>
     <t>Trạng thái</t>
   </si>
   <si>
     <t>Đức</t>
   </si>
   <si>
-    <t>Backend &amp; AI Specialist</t>
-  </si>
-  <si>
-    <t>* Tối ưu hóa logic Gemini và OCR.* Quản lý kết nối Supabase từ phía Server.* Hỗ trợ các thành viên khác kết nối API.</t>
-  </si>
-  <si>
-    <t>Đã xong 80%</t>
-  </si>
-  <si>
     <t>Khang</t>
   </si>
   <si>
-    <t>Frontend Developer (UI/UX)</t>
-  </si>
-  <si>
-    <t>* Xây dựng giao diện Next.js theo mẫu đã thiết kế.* Viết logic bắt sự kiện onPaste và xử lý hiển thị ảnh tạm thời.* Gọi API /chat và /ocr từ phía người dùng.</t>
-  </si>
-  <si>
     <t>Sắp thực hiện</t>
   </si>
   <si>
     <t>Lý</t>
   </si>
   <si>
-    <t>Auth &amp; System Admin</t>
-  </si>
-  <si>
-    <t>* Thiết lập Google Cloud Console (Lấy Client ID/Secret).* Tích hợp Supabase Auth (Đăng nhập Google) vào Frontend.* Đảm bảo luồng user_id được truyền chính xác để lưu lịch sử.</t>
-  </si>
-  <si>
     <t>Đang thực hiện</t>
   </si>
   <si>
     <t>Kiệt</t>
   </si>
   <si>
-    <t>QA Tester &amp; DevOps</t>
-  </si>
-  <si>
-    <t>* Triển khai dự án lên máy ảo (Render cho Backend, Vercel cho Frontend).* Quản lý bảo mật file .env trên môi trường Production.* Viết tài liệu hướng dẫn (README) và thực hiện các kịch bản test lỗi.</t>
-  </si>
-  <si>
     <t>Hạng mục</t>
   </si>
   <si>
@@ -95,9 +65,6 @@
     <t>Chốt Tech Stack</t>
   </si>
   <si>
-    <t>Next.js, FastAPI, Supabase, Gemini API</t>
-  </si>
-  <si>
     <t>Hoàn thành</t>
   </si>
   <si>
@@ -110,24 +77,15 @@
     <t>Git &amp; GitHub</t>
   </si>
   <si>
-    <t>Khởi tạo repo, .gitignore, kết nối GitHub</t>
-  </si>
-  <si>
     <t>Backend</t>
   </si>
   <si>
     <t>Môi trường ảo</t>
   </si>
   <si>
-    <t>Thiết lập venv</t>
-  </si>
-  <si>
     <t>Cài đặt thư viện</t>
   </si>
   <si>
-    <t>Cài đặt core libraries (FastAPI, Gemini, Pillow, v.v.)</t>
-  </si>
-  <si>
     <t>Xử lý lỗi C++</t>
   </si>
   <si>
@@ -137,9 +95,6 @@
     <t>Logic xử lý (main.py)</t>
   </si>
   <si>
-    <t>Chatbot và OCR (đọc ảnh)</t>
-  </si>
-  <si>
     <t>Database</t>
   </si>
   <si>
@@ -161,9 +116,6 @@
     <t>Backend &lt;-&gt; Database</t>
   </si>
   <si>
-    <t>Kiểm thử lưu trữ tin nhắn thực tế</t>
-  </si>
-  <si>
     <t>Authentication</t>
   </si>
   <si>
@@ -182,21 +134,6 @@
     <t>Xây dựng UI với Tailwind CSS</t>
   </si>
   <si>
-    <t>Xử lý Clipboard (onPaste)</t>
-  </si>
-  <si>
-    <t>Dán ảnh trực tiếp từ clipboard</t>
-  </si>
-  <si>
-    <t>Kết nối API</t>
-  </si>
-  <si>
-    <t>Tích hợp Đăng nhập</t>
-  </si>
-  <si>
-    <t>Nút Login Google và quản lý user_id</t>
-  </si>
-  <si>
     <t>Deployment</t>
   </si>
   <si>
@@ -227,7 +164,81 @@
     <t>Kiểm tra các trường hợp biên, lỗi AI, auth</t>
   </si>
   <si>
-    <t>Liên kết UI với Backend (/chat, /ocr)</t>
+    <t>Nhiệm vụ chi tiết</t>
+  </si>
+  <si>
+    <t>Backend &amp; AI</t>
+  </si>
+  <si>
+    <t>* Tối ưu hóa logic Gemini và OCR. * Quản lý kết nối Supabase từ phía Server.</t>
+  </si>
+  <si>
+    <t>Frontend (UI/UX)</t>
+  </si>
+  <si>
+    <t>* Xây dựng giao diện Next.js. * Viết logic bắt sự kiện onPaste.</t>
+  </si>
+  <si>
+    <t>Auth &amp; Admin</t>
+  </si>
+  <si>
+    <t>* Tích hợp Supabase Auth vào Frontend. * Đảm bảo luồng user_id truyền chính xác.</t>
+  </si>
+  <si>
+    <t>QA &amp; DevOps</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Triển khai dự án lên Hugging Face Spaces.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> * Quản lý bảo mật Key trong mục Secrets.</t>
+    </r>
+  </si>
+  <si>
+    <t>Đã xong 95%</t>
+  </si>
+  <si>
+    <t>"Next.js, FastAPI, Supabase, Gemini API"</t>
+  </si>
+  <si>
+    <t>"Khởi tạo repo, .gitignore, kết nối GitHub"</t>
+  </si>
+  <si>
+    <t>Thiết lập venv (Đã xử lý Python 3.14/3.13)</t>
+  </si>
+  <si>
+    <t>Cài đặt core libraries (Xử lý xong lỗi Supabase/Pyiceberg)</t>
+  </si>
+  <si>
+    <t>Hoàn thiện API Chat và OCR</t>
+  </si>
+  <si>
+    <t>Tích hợp logic lưu trữ tin nhắn vào main.py</t>
+  </si>
+  <si>
+    <t>Đang đẩy lên Hugging Face Spaces (Docker)</t>
+  </si>
+  <si>
+    <t>Thiết lập Secrets (API Key) trên Hugging Face</t>
   </si>
 </sst>
 </file>
@@ -255,14 +266,15 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -271,24 +283,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FF8ED7DD"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -312,15 +312,39 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top/>
+      <bottom style="thin">
         <color indexed="64"/>
-      </top>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -333,22 +357,22 @@
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -569,82 +593,82 @@
   <cols>
     <col min="1" max="1" width="10.6640625" customWidth="1"/>
     <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="168.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="179.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="B3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="B4" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" spans="1:5" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="1"/>
-    </row>
-    <row r="5" spans="1:5" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>11</v>
+      <c r="B5" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="E5" s="1"/>
     </row>
@@ -655,7 +679,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE36B8C3-337D-4F75-BEDD-54A03575897A}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.109375" customWidth="1"/>
@@ -664,285 +688,303 @@
     <col min="4" max="4" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C6" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D7" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C8" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D9" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D10" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="B11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D12" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="4" t="s">
+      <c r="D15" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="B17" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="C17" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="D17" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C18" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B10" s="4" t="s">
+      <c r="D18" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C19" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="D19" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B20" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C20" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>67</v>
-      </c>
       <c r="D20" s="6" t="s">
-        <v>11</v>
-      </c>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Enhance accessibility and responsiveness in chat UI; update Tailwind configuration and remove unused PostCSS config
</commit_message>
<xml_diff>
--- a/Chia nhiệm vụ dự án MentorPro.xlsx
+++ b/Chia nhiệm vụ dự án MentorPro.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MentorPro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{782FD814-F13C-4852-A6A2-8C234B0E133E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5A0682C-7701-428F-A269-85381187290F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chia nhiệm vụ dự án MentorPro" sheetId="1" r:id="rId1"/>
@@ -274,7 +274,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -283,7 +283,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF8ED7DD"/>
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -354,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -364,10 +382,22 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -593,7 +623,7 @@
   <cols>
     <col min="1" max="1" width="10.6640625" customWidth="1"/>
     <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="179.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="76.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -684,7 +714,7 @@
   <cols>
     <col min="1" max="1" width="16.109375" customWidth="1"/>
     <col min="2" max="2" width="13.33203125" customWidth="1"/>
-    <col min="3" max="3" width="52.33203125" customWidth="1"/>
+    <col min="3" max="3" width="49.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -703,268 +733,268 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="7" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="7" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="8" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="8" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="10" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>